<commit_message>
Actualizar Excel y script con observaciones REVISAR
Co-authored-by: JordanS2209 <213678298+JordanS2209@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/factura_con_iva.xlsx
+++ b/factura_con_iva.xlsx
@@ -666,7 +666,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>REVISAR: los totales calculados no coinciden con los impresos; faltan líneas por transcribir o validar en las fotos.</t>
+          <t>REVISAR: los totales calculados no coinciden con los impresos (subtotal 287.39, IVA 43.11, total 330.50); faltan líneas por transcribir o validar en las fotos.</t>
         </is>
       </c>
     </row>
@@ -681,7 +681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -725,14 +725,42 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Se necesita la lista del pedido original para detectar faltantes.</t>
+          <t>No se pudo transcribir la lista solicitada (imágenes 8-11) desde el contenido accesible en este entorno.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Nota</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>La comparación se basa en la factura recibida y la lista proporcionada. Las unidades por caja/paquete requieren confirmación cuando no coinciden.</t>
         </is>
       </c>
     </row>

</xml_diff>